<commit_message>
Refresh Phase 6B–6D diagnostics from Phase 6F store export pipeline run.
Align adjacent-path, ATS, graph, active-learning, and calibration eligibility artifacts with the latest store 772 reporting export.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Diagnostics/phase6d01_dag_active_learning_adjacent_calibration/ACTIVE_LEARNING_TOP_100_REVIEW.xlsx
+++ b/Diagnostics/phase6d01_dag_active_learning_adjacent_calibration/ACTIVE_LEARNING_TOP_100_REVIEW.xlsx
@@ -24,13 +24,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -41,7 +44,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +52,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -424,122 +436,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -10364,122 +10376,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -20304,122 +20316,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -20440,122 +20452,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -29984,122 +29996,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -31888,122 +31900,122 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>store_number</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>promotion_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sku_number</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>department</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>category</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>active_learning_score</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>active_learning_rank</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>active_learning_reason</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>expected_information_gain</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>human_review_question</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>which_model_component_will_learn</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>priority_bucket</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>dag_state_missingness_risk_score</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>adjacent_path_use_policy</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>adjacent_confidence_calibrated</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>final_governed_action_label</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>final_governed_order_units</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>model_expected_units_total_promo</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>adjacent_expected_units</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>available_to_sell_confidence_score</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>weak_history_flag</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>new_line_flag</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>long_tail_sku_flag</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="X1" s="1" t="inlineStr">
         <is>
           <t>mission_sku_score</t>
         </is>
@@ -41828,12 +41840,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>section</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>text</t>
         </is>
@@ -41890,12 +41902,12 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>field</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>allowed_values</t>
         </is>

</xml_diff>